<commit_message>
Versión v1 Observatori Calp
</commit_message>
<xml_diff>
--- a/data/DB_Dashboard.xlsx
+++ b/data/DB_Dashboard.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jmari\Desktop\Observatorio Calp\observatorio_calp\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{57E54697-B080-4C1B-B2B8-7CC63FE6A5E3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{454D9A31-421E-4B80-B3A6-2193DD68ED30}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{A3E3E45F-D34A-4772-8FFC-37BF922E3DDC}"/>
   </bookViews>
@@ -43,7 +43,7 @@
     <author>tc={86248D9D-A426-4266-983B-342EA897A500}</author>
   </authors>
   <commentList>
-    <comment ref="M30" authorId="0" shapeId="0" xr:uid="{86248D9D-A426-4266-983B-342EA897A500}">
+    <comment ref="M31" authorId="0" shapeId="0" xr:uid="{86248D9D-A426-4266-983B-342EA897A500}">
       <text>
         <t>[Comentario encadenado]
 Su versión de Excel le permite leer este comentario encadenado; sin embargo, las ediciones que se apliquen se quitarán si el archivo se abre en una versión más reciente de Excel. Más información: https://go.microsoft.com/fwlink/?linkid=870924
@@ -56,7 +56,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="668" uniqueCount="340">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="679" uniqueCount="347">
   <si>
     <t>Año</t>
   </si>
@@ -1463,6 +1463,27 @@
   </si>
   <si>
     <t>ETIS - Residuos reciclados por residentes respecto al total</t>
+  </si>
+  <si>
+    <t>Número de turistas o visitantes extranjeros que visitaron Calp durante el último año.</t>
+  </si>
+  <si>
+    <t>Número de turistas o visitantes nacionales que visitaron Calp durante el último año.</t>
+  </si>
+  <si>
+    <t>WTO - Estacionalidad turística</t>
+  </si>
+  <si>
+    <t>Recuendo de turistas extranjero que visitaron Calp por mes.</t>
+  </si>
+  <si>
+    <t>Recuendo de turistas nacionales que visitaron Calp por mes.</t>
+  </si>
+  <si>
+    <t>Nº de turistas nacionales que visitaron Calp en el último año. Datos mensuales</t>
+  </si>
+  <si>
+    <t>Nº de turistas extranjeros que visitaron Calp en el último año. Datos mensuales</t>
   </si>
 </sst>
 </file>
@@ -1558,7 +1579,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="11">
+  <borders count="12">
     <border>
       <left/>
       <right/>
@@ -1686,13 +1707,24 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="7" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="47">
+  <cellXfs count="48">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1802,6 +1834,7 @@
     <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Hipervínculo" xfId="1" builtinId="8"/>
@@ -1809,6 +1842,12 @@
     <cellStyle name="Porcentaje" xfId="2" builtinId="5"/>
   </cellStyles>
   <dxfs count="35">
+    <dxf>
+      <numFmt numFmtId="164" formatCode="0.0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="0.0"/>
+    </dxf>
     <dxf>
       <font>
         <b val="0"/>
@@ -1982,12 +2021,6 @@
       </font>
     </dxf>
     <dxf>
-      <numFmt numFmtId="164" formatCode="0.0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="0.0"/>
-    </dxf>
-    <dxf>
       <numFmt numFmtId="3" formatCode="#,##0"/>
     </dxf>
     <dxf>
@@ -2556,14 +2589,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{72A2E2F1-7CAD-4C76-BEFF-2442C0A18302}" name="Dashboard" displayName="Dashboard" ref="A1:O52" totalsRowShown="0" headerRowDxfId="34" dataDxfId="32" headerRowBorderDxfId="33" tableBorderDxfId="31" totalsRowBorderDxfId="30">
-  <autoFilter ref="A1:O52" xr:uid="{72A2E2F1-7CAD-4C76-BEFF-2442C0A18302}">
-    <filterColumn colId="4">
-      <filters>
-        <filter val="Gestión de residuos"/>
-      </filters>
-    </filterColumn>
-  </autoFilter>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{72A2E2F1-7CAD-4C76-BEFF-2442C0A18302}" name="Dashboard" displayName="Dashboard" ref="A1:O53" totalsRowShown="0" headerRowDxfId="34" dataDxfId="32" headerRowBorderDxfId="33" tableBorderDxfId="31" totalsRowBorderDxfId="30">
+  <autoFilter ref="A1:O53" xr:uid="{72A2E2F1-7CAD-4C76-BEFF-2442C0A18302}"/>
   <tableColumns count="15">
     <tableColumn id="1" xr3:uid="{1793D8B9-1834-4672-94E2-370894E55593}" name="Año" dataDxfId="29"/>
     <tableColumn id="12" xr3:uid="{2FF65C8B-F0E1-459C-B72F-3A1A5329FDAB}" name="ETIS" dataDxfId="28"/>
@@ -2595,25 +2622,29 @@
     <tableColumn id="2" xr3:uid="{B343196D-F313-4338-A33E-C35CA22E1037}" name="1. Turistas extranjeros que visitaron Calp" dataDxfId="14"/>
     <tableColumn id="3" xr3:uid="{7694471A-5A27-4BAB-9627-5B49B697400E}" name="1. Turistas nacionales que visitaron Calp" dataDxfId="13"/>
     <tableColumn id="4" xr3:uid="{1BAEF350-378C-40C2-820B-759FCF4ED388}" name="1. Total turistas" dataDxfId="12"/>
-    <tableColumn id="5" xr3:uid="{A35DAE71-EE4A-4EC9-8460-F2F26963F5A2}" name="2.% Turistas extranjeros que visitaron Calp" dataDxfId="11"/>
-    <tableColumn id="6" xr3:uid="{77257F63-E741-45A0-A7C8-573D91BC35FA}" name="2. % Turistas nacionales que visitaron Calp" dataDxfId="10"/>
+    <tableColumn id="5" xr3:uid="{A35DAE71-EE4A-4EC9-8460-F2F26963F5A2}" name="2.% Turistas extranjeros que visitaron Calp" dataDxfId="0">
+      <calculatedColumnFormula>Turistas[[#This Row],[1. Turistas extranjeros que visitaron Calp]]/Turistas[[#This Row],[1. Total turistas]]</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="6" xr3:uid="{77257F63-E741-45A0-A7C8-573D91BC35FA}" name="2. % Turistas nacionales que visitaron Calp" dataDxfId="1">
+      <calculatedColumnFormula>Turistas[[#This Row],[1. Turistas nacionales que visitaron Calp]]/Turistas[[#This Row],[1. Total turistas]]</calculatedColumnFormula>
+    </tableColumn>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{32B811EC-84D2-45FC-891C-7E090EB6CBCD}" name="Alojamientos" displayName="Alojamientos" ref="A1:H9" totalsRowShown="0" headerRowDxfId="9" dataDxfId="8">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{32B811EC-84D2-45FC-891C-7E090EB6CBCD}" name="Alojamientos" displayName="Alojamientos" ref="A1:H9" totalsRowShown="0" headerRowDxfId="11" dataDxfId="10">
   <autoFilter ref="A1:H9" xr:uid="{32B811EC-84D2-45FC-891C-7E090EB6CBCD}"/>
   <tableColumns count="8">
-    <tableColumn id="1" xr3:uid="{07BCC607-7EEB-4361-B136-CCDA8E5F70BE}" name="Tipo" dataDxfId="7"/>
-    <tableColumn id="8" xr3:uid="{0871BF09-A2EB-42F4-86E2-C14CDB481EC8}" name="Año" dataDxfId="6"/>
-    <tableColumn id="2" xr3:uid="{B1AB5E11-B4CF-48BB-A35C-C459F9489AB4}" name="Establecimientos" dataDxfId="5"/>
-    <tableColumn id="3" xr3:uid="{ACC63EB1-5B06-4BEE-9E7E-B340C9BD2498}" name="Plazas" dataDxfId="4"/>
-    <tableColumn id="4" xr3:uid="{03DB75FF-9B48-49D9-9D17-D4363A5A9025}" name="Habitaciones" dataDxfId="3"/>
-    <tableColumn id="5" xr3:uid="{B55E2CBA-9D33-447F-AFD9-B5ED8123A040}" name="Parcelas" dataDxfId="2"/>
-    <tableColumn id="6" xr3:uid="{18A9F2D6-F247-4306-843D-3BC9A08F8F16}" name="% alojamientos" dataDxfId="1" dataCellStyle="Porcentaje"/>
-    <tableColumn id="7" xr3:uid="{0CA9FABA-AC27-4D35-A37F-5ADFC3A1E28A}" name="% plazas" dataDxfId="0" dataCellStyle="Porcentaje">
+    <tableColumn id="1" xr3:uid="{07BCC607-7EEB-4361-B136-CCDA8E5F70BE}" name="Tipo" dataDxfId="9"/>
+    <tableColumn id="8" xr3:uid="{0871BF09-A2EB-42F4-86E2-C14CDB481EC8}" name="Año" dataDxfId="8"/>
+    <tableColumn id="2" xr3:uid="{B1AB5E11-B4CF-48BB-A35C-C459F9489AB4}" name="Establecimientos" dataDxfId="7"/>
+    <tableColumn id="3" xr3:uid="{ACC63EB1-5B06-4BEE-9E7E-B340C9BD2498}" name="Plazas" dataDxfId="6"/>
+    <tableColumn id="4" xr3:uid="{03DB75FF-9B48-49D9-9D17-D4363A5A9025}" name="Habitaciones" dataDxfId="5"/>
+    <tableColumn id="5" xr3:uid="{B55E2CBA-9D33-447F-AFD9-B5ED8123A040}" name="Parcelas" dataDxfId="4"/>
+    <tableColumn id="6" xr3:uid="{18A9F2D6-F247-4306-843D-3BC9A08F8F16}" name="% alojamientos" dataDxfId="3" dataCellStyle="Porcentaje"/>
+    <tableColumn id="7" xr3:uid="{0CA9FABA-AC27-4D35-A37F-5ADFC3A1E28A}" name="% plazas" dataDxfId="2" dataCellStyle="Porcentaje">
       <calculatedColumnFormula>D2/D$9</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -2938,7 +2969,7 @@
 
 <file path=xl/threadedComments/threadedComment1.xml><?xml version="1.0" encoding="utf-8"?>
 <ThreadedComments xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <threadedComment ref="M30" dT="2025-12-11T16:46:50.50" personId="{AB9528B7-6643-4F77-B76C-533514F2F00F}" id="{86248D9D-A426-4266-983B-342EA897A500}">
+  <threadedComment ref="M31" dT="2025-12-11T16:46:50.50" personId="{AB9528B7-6643-4F77-B76C-533514F2F00F}" id="{86248D9D-A426-4266-983B-342EA897A500}">
     <text>Preguntar a Paula si tenim este dato</text>
   </threadedComment>
 </ThreadedComments>
@@ -2946,7 +2977,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{27BA13B8-EC56-4433-A73B-150D55368D4D}">
-  <dimension ref="A1:O52"/>
+  <dimension ref="A1:O53"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16.8" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="1" max="2" width="11.5546875" style="37"/>
@@ -3012,7 +3043,7 @@
         <v>163</v>
       </c>
     </row>
-    <row r="2" spans="1:15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:15" x14ac:dyDescent="0.4">
       <c r="A2" s="24">
         <v>2024</v>
       </c>
@@ -3059,7 +3090,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="3" spans="1:15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:15" x14ac:dyDescent="0.4">
       <c r="A3" s="5">
         <v>2024</v>
       </c>
@@ -3104,7 +3135,7 @@
       </c>
       <c r="O3" s="11"/>
     </row>
-    <row r="4" spans="1:15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:15" x14ac:dyDescent="0.4">
       <c r="A4" s="5">
         <v>2024</v>
       </c>
@@ -3149,7 +3180,7 @@
       </c>
       <c r="O4" s="8"/>
     </row>
-    <row r="5" spans="1:15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:15" x14ac:dyDescent="0.4">
       <c r="A5" s="5">
         <v>2024</v>
       </c>
@@ -3194,7 +3225,7 @@
       </c>
       <c r="O5" s="6"/>
     </row>
-    <row r="6" spans="1:15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:15" x14ac:dyDescent="0.4">
       <c r="A6" s="5">
         <v>2024</v>
       </c>
@@ -3239,7 +3270,7 @@
       </c>
       <c r="O6" s="6"/>
     </row>
-    <row r="7" spans="1:15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:15" x14ac:dyDescent="0.4">
       <c r="A7" s="24">
         <v>2024</v>
       </c>
@@ -3286,7 +3317,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="8" spans="1:15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:15" x14ac:dyDescent="0.4">
       <c r="A8" s="24">
         <v>2024</v>
       </c>
@@ -3333,7 +3364,7 @@
         <v>212</v>
       </c>
     </row>
-    <row r="9" spans="1:15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:15" x14ac:dyDescent="0.4">
       <c r="A9" s="24">
         <v>2024</v>
       </c>
@@ -3378,7 +3409,7 @@
       </c>
       <c r="O9" s="29"/>
     </row>
-    <row r="10" spans="1:15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:15" x14ac:dyDescent="0.4">
       <c r="A10" s="24">
         <v>2024</v>
       </c>
@@ -3423,7 +3454,7 @@
       </c>
       <c r="O10" s="29"/>
     </row>
-    <row r="11" spans="1:15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:15" x14ac:dyDescent="0.4">
       <c r="A11" s="24">
         <v>2024</v>
       </c>
@@ -3470,7 +3501,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="12" spans="1:15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:15" x14ac:dyDescent="0.4">
       <c r="A12" s="24">
         <v>2024</v>
       </c>
@@ -3517,7 +3548,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="13" spans="1:15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:15" x14ac:dyDescent="0.4">
       <c r="A13" s="24">
         <v>2024</v>
       </c>
@@ -3564,7 +3595,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="14" spans="1:15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="14" spans="1:15" x14ac:dyDescent="0.4">
       <c r="A14" s="24">
         <v>2024</v>
       </c>
@@ -3611,7 +3642,7 @@
         <v>185</v>
       </c>
     </row>
-    <row r="15" spans="1:15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="15" spans="1:15" x14ac:dyDescent="0.4">
       <c r="A15" s="24">
         <v>2024</v>
       </c>
@@ -3656,7 +3687,7 @@
       </c>
       <c r="O15" s="42"/>
     </row>
-    <row r="16" spans="1:15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="16" spans="1:15" x14ac:dyDescent="0.4">
       <c r="A16" s="24">
         <v>2024</v>
       </c>
@@ -3701,7 +3732,7 @@
       </c>
       <c r="O16" s="42"/>
     </row>
-    <row r="17" spans="1:15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="17" spans="1:15" x14ac:dyDescent="0.4">
       <c r="A17" s="24">
         <v>2024</v>
       </c>
@@ -3746,153 +3777,153 @@
       </c>
       <c r="O17" s="42"/>
     </row>
-    <row r="18" spans="1:15" hidden="1" x14ac:dyDescent="0.4">
-      <c r="A18" s="18">
-        <v>2024</v>
-      </c>
-      <c r="B18" s="19" t="s">
+    <row r="18" spans="1:15" x14ac:dyDescent="0.4">
+      <c r="A18" s="24">
+        <v>2024</v>
+      </c>
+      <c r="B18" s="25" t="s">
         <v>123</v>
       </c>
-      <c r="C18" s="20" t="s">
+      <c r="C18" s="26" t="s">
         <v>20</v>
       </c>
-      <c r="D18" s="20">
+      <c r="D18" s="26">
         <v>4</v>
       </c>
-      <c r="E18" s="20" t="s">
+      <c r="E18" s="26" t="s">
         <v>23</v>
       </c>
-      <c r="F18" s="20" t="s">
+      <c r="F18" s="26" t="s">
+        <v>340</v>
+      </c>
+      <c r="G18" s="26" t="s">
+        <v>342</v>
+      </c>
+      <c r="H18" s="26" t="s">
+        <v>64</v>
+      </c>
+      <c r="I18" s="26" t="s">
+        <v>271</v>
+      </c>
+      <c r="J18" s="26" t="s">
+        <v>11</v>
+      </c>
+      <c r="K18" s="27" t="s">
+        <v>17</v>
+      </c>
+      <c r="L18" s="26" t="s">
+        <v>343</v>
+      </c>
+      <c r="M18" s="26" t="s">
+        <v>346</v>
+      </c>
+      <c r="N18" s="32">
+        <v>247964</v>
+      </c>
+      <c r="O18" s="29" t="s">
         <v>123</v>
       </c>
-      <c r="G18" s="20" t="s">
+    </row>
+    <row r="19" spans="1:15" x14ac:dyDescent="0.4">
+      <c r="A19" s="47">
+        <v>2024</v>
+      </c>
+      <c r="B19" s="25" t="s">
         <v>123</v>
       </c>
-      <c r="H18" s="20" t="s">
+      <c r="C19" s="26" t="s">
+        <v>20</v>
+      </c>
+      <c r="D19" s="26">
+        <v>4</v>
+      </c>
+      <c r="E19" s="26" t="s">
+        <v>23</v>
+      </c>
+      <c r="F19" s="26" t="s">
+        <v>341</v>
+      </c>
+      <c r="G19" s="26" t="s">
+        <v>342</v>
+      </c>
+      <c r="H19" s="26" t="s">
+        <v>64</v>
+      </c>
+      <c r="I19" s="26" t="s">
+        <v>271</v>
+      </c>
+      <c r="J19" s="26" t="s">
+        <v>11</v>
+      </c>
+      <c r="K19" s="27" t="s">
+        <v>17</v>
+      </c>
+      <c r="L19" s="26" t="s">
+        <v>344</v>
+      </c>
+      <c r="M19" s="26" t="s">
+        <v>345</v>
+      </c>
+      <c r="N19" s="32">
+        <v>310709</v>
+      </c>
+      <c r="O19" s="25" t="s">
         <v>123</v>
       </c>
-      <c r="I18" s="20" t="s">
+    </row>
+    <row r="20" spans="1:15" x14ac:dyDescent="0.4">
+      <c r="A20" s="5">
+        <v>2024</v>
+      </c>
+      <c r="B20" s="6" t="s">
+        <v>236</v>
+      </c>
+      <c r="C20" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="D20" s="7">
+        <v>5</v>
+      </c>
+      <c r="E20" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="F20" s="7" t="s">
+        <v>237</v>
+      </c>
+      <c r="G20" s="7" t="s">
+        <v>238</v>
+      </c>
+      <c r="H20" s="7" t="s">
+        <v>232</v>
+      </c>
+      <c r="I20" s="7" t="s">
+        <v>233</v>
+      </c>
+      <c r="J20" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="K20" s="8" t="s">
+        <v>235</v>
+      </c>
+      <c r="L20" s="7" t="s">
+        <v>234</v>
+      </c>
+      <c r="M20" s="7" t="s">
+        <v>240</v>
+      </c>
+      <c r="N20" s="9" t="s">
         <v>123</v>
       </c>
-      <c r="J18" s="20" t="s">
-        <v>123</v>
-      </c>
-      <c r="K18" s="21" t="s">
-        <v>123</v>
-      </c>
-      <c r="L18" s="20" t="s">
-        <v>123</v>
-      </c>
-      <c r="M18" s="20" t="s">
-        <v>123</v>
-      </c>
-      <c r="N18" s="22" t="s">
-        <v>123</v>
-      </c>
-      <c r="O18" s="23" t="s">
-        <v>123</v>
-      </c>
-    </row>
-    <row r="19" spans="1:15" hidden="1" x14ac:dyDescent="0.4">
-      <c r="A19" s="5">
-        <v>2024</v>
-      </c>
-      <c r="B19" s="6" t="s">
-        <v>236</v>
-      </c>
-      <c r="C19" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="D19" s="7">
-        <v>5</v>
-      </c>
-      <c r="E19" s="7" t="s">
-        <v>24</v>
-      </c>
-      <c r="F19" s="7" t="s">
-        <v>237</v>
-      </c>
-      <c r="G19" s="7" t="s">
-        <v>238</v>
-      </c>
-      <c r="H19" s="7" t="s">
-        <v>232</v>
-      </c>
-      <c r="I19" s="7" t="s">
-        <v>233</v>
-      </c>
-      <c r="J19" s="7" t="s">
-        <v>11</v>
-      </c>
-      <c r="K19" s="8" t="s">
-        <v>235</v>
-      </c>
-      <c r="L19" s="7" t="s">
-        <v>234</v>
-      </c>
-      <c r="M19" s="7" t="s">
-        <v>240</v>
-      </c>
-      <c r="N19" s="9" t="s">
-        <v>123</v>
-      </c>
-      <c r="O19" s="8" t="s">
+      <c r="O20" s="8" t="s">
         <v>239</v>
       </c>
     </row>
-    <row r="20" spans="1:15" hidden="1" x14ac:dyDescent="0.4">
-      <c r="A20" s="24">
-        <v>2024</v>
-      </c>
-      <c r="B20" s="25" t="s">
+    <row r="21" spans="1:15" x14ac:dyDescent="0.4">
+      <c r="A21" s="24">
+        <v>2024</v>
+      </c>
+      <c r="B21" s="25" t="s">
         <v>139</v>
-      </c>
-      <c r="C20" s="26" t="s">
-        <v>20</v>
-      </c>
-      <c r="D20" s="26">
-        <v>6</v>
-      </c>
-      <c r="E20" s="26" t="s">
-        <v>25</v>
-      </c>
-      <c r="F20" s="26" t="s">
-        <v>140</v>
-      </c>
-      <c r="G20" s="26" t="s">
-        <v>203</v>
-      </c>
-      <c r="H20" s="26" t="s">
-        <v>141</v>
-      </c>
-      <c r="I20" s="26" t="s">
-        <v>141</v>
-      </c>
-      <c r="J20" s="26" t="s">
-        <v>143</v>
-      </c>
-      <c r="K20" s="27" t="s">
-        <v>12</v>
-      </c>
-      <c r="L20" s="26" t="s">
-        <v>144</v>
-      </c>
-      <c r="M20" s="26" t="s">
-        <v>142</v>
-      </c>
-      <c r="N20" s="28">
-        <v>68.89</v>
-      </c>
-      <c r="O20" s="29" t="s">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="21" spans="1:15" ht="18" hidden="1" x14ac:dyDescent="0.4">
-      <c r="A21" s="24">
-        <v>2024</v>
-      </c>
-      <c r="B21" s="25" t="s">
-        <v>148</v>
       </c>
       <c r="C21" s="26" t="s">
         <v>20</v>
@@ -3904,42 +3935,42 @@
         <v>25</v>
       </c>
       <c r="F21" s="26" t="s">
-        <v>149</v>
+        <v>140</v>
       </c>
       <c r="G21" s="26" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="H21" s="26" t="s">
-        <v>57</v>
+        <v>141</v>
       </c>
       <c r="I21" s="26" t="s">
-        <v>150</v>
+        <v>141</v>
       </c>
       <c r="J21" s="26" t="s">
-        <v>11</v>
+        <v>143</v>
       </c>
       <c r="K21" s="27" t="s">
-        <v>154</v>
+        <v>12</v>
       </c>
       <c r="L21" s="26" t="s">
-        <v>153</v>
+        <v>144</v>
       </c>
       <c r="M21" s="26" t="s">
-        <v>156</v>
+        <v>142</v>
       </c>
       <c r="N21" s="28">
-        <v>6.59</v>
+        <v>68.89</v>
       </c>
       <c r="O21" s="29" t="s">
-        <v>155</v>
-      </c>
-    </row>
-    <row r="22" spans="1:15" ht="18" hidden="1" x14ac:dyDescent="0.4">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="22" spans="1:15" ht="18" x14ac:dyDescent="0.4">
       <c r="A22" s="24">
         <v>2024</v>
       </c>
       <c r="B22" s="25" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="C22" s="26" t="s">
         <v>20</v>
@@ -3969,24 +4000,24 @@
         <v>154</v>
       </c>
       <c r="L22" s="26" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="M22" s="26" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="N22" s="28">
-        <v>12.02</v>
+        <v>6.59</v>
       </c>
       <c r="O22" s="29" t="s">
         <v>155</v>
       </c>
     </row>
-    <row r="23" spans="1:15" ht="18" hidden="1" x14ac:dyDescent="0.4">
+    <row r="23" spans="1:15" ht="18" x14ac:dyDescent="0.4">
       <c r="A23" s="24">
         <v>2024</v>
       </c>
       <c r="B23" s="25" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="C23" s="26" t="s">
         <v>20</v>
@@ -4016,63 +4047,63 @@
         <v>154</v>
       </c>
       <c r="L23" s="26" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="M23" s="26" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="N23" s="28">
-        <v>9.56</v>
+        <v>12.02</v>
       </c>
       <c r="O23" s="29" t="s">
         <v>155</v>
       </c>
     </row>
-    <row r="24" spans="1:15" x14ac:dyDescent="0.4">
+    <row r="24" spans="1:15" ht="18" x14ac:dyDescent="0.4">
       <c r="A24" s="24">
         <v>2024</v>
       </c>
       <c r="B24" s="25" t="s">
-        <v>48</v>
+        <v>146</v>
       </c>
       <c r="C24" s="26" t="s">
         <v>20</v>
       </c>
       <c r="D24" s="26">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E24" s="26" t="s">
-        <v>18</v>
+        <v>25</v>
       </c>
       <c r="F24" s="26" t="s">
-        <v>37</v>
+        <v>149</v>
       </c>
       <c r="G24" s="26" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="H24" s="26" t="s">
-        <v>38</v>
+        <v>57</v>
       </c>
       <c r="I24" s="26" t="s">
-        <v>40</v>
+        <v>150</v>
       </c>
       <c r="J24" s="26" t="s">
         <v>11</v>
       </c>
       <c r="K24" s="27" t="s">
-        <v>41</v>
+        <v>154</v>
       </c>
       <c r="L24" s="26" t="s">
-        <v>45</v>
+        <v>152</v>
       </c>
       <c r="M24" s="26" t="s">
-        <v>113</v>
+        <v>158</v>
       </c>
       <c r="N24" s="28">
-        <v>36.78</v>
+        <v>9.56</v>
       </c>
       <c r="O24" s="29" t="s">
-        <v>54</v>
+        <v>155</v>
       </c>
     </row>
     <row r="25" spans="1:15" x14ac:dyDescent="0.4">
@@ -4080,7 +4111,7 @@
         <v>2024</v>
       </c>
       <c r="B25" s="25" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="C25" s="26" t="s">
         <v>20</v>
@@ -4095,7 +4126,7 @@
         <v>37</v>
       </c>
       <c r="G25" s="26" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="H25" s="26" t="s">
         <v>38</v>
@@ -4110,13 +4141,13 @@
         <v>41</v>
       </c>
       <c r="L25" s="26" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="M25" s="26" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="N25" s="28">
-        <v>34.18</v>
+        <v>36.78</v>
       </c>
       <c r="O25" s="29" t="s">
         <v>54</v>
@@ -4127,7 +4158,7 @@
         <v>2024</v>
       </c>
       <c r="B26" s="25" t="s">
-        <v>136</v>
+        <v>47</v>
       </c>
       <c r="C26" s="26" t="s">
         <v>20</v>
@@ -4139,10 +4170,10 @@
         <v>18</v>
       </c>
       <c r="F26" s="26" t="s">
-        <v>42</v>
+        <v>37</v>
       </c>
       <c r="G26" s="26" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="H26" s="26" t="s">
         <v>38</v>
@@ -4154,19 +4185,19 @@
         <v>11</v>
       </c>
       <c r="K26" s="27" t="s">
-        <v>12</v>
+        <v>41</v>
       </c>
       <c r="L26" s="26" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="M26" s="26" t="s">
-        <v>52</v>
+        <v>112</v>
       </c>
       <c r="N26" s="28">
-        <v>50.85</v>
+        <v>34.18</v>
       </c>
       <c r="O26" s="29" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
     </row>
     <row r="27" spans="1:15" x14ac:dyDescent="0.4">
@@ -4174,7 +4205,7 @@
         <v>2024</v>
       </c>
       <c r="B27" s="25" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="C27" s="26" t="s">
         <v>20</v>
@@ -4185,11 +4216,11 @@
       <c r="E27" s="26" t="s">
         <v>18</v>
       </c>
-      <c r="F27" s="46" t="s">
-        <v>336</v>
+      <c r="F27" s="26" t="s">
+        <v>42</v>
       </c>
       <c r="G27" s="26" t="s">
-        <v>339</v>
+        <v>199</v>
       </c>
       <c r="H27" s="26" t="s">
         <v>38</v>
@@ -4201,19 +4232,19 @@
         <v>11</v>
       </c>
       <c r="K27" s="27" t="s">
-        <v>43</v>
+        <v>12</v>
       </c>
       <c r="L27" s="26" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="M27" s="26" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="N27" s="28">
-        <v>2.1</v>
+        <v>50.85</v>
       </c>
       <c r="O27" s="29" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="28" spans="1:15" x14ac:dyDescent="0.4">
@@ -4221,7 +4252,7 @@
         <v>2024</v>
       </c>
       <c r="B28" s="25" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="C28" s="26" t="s">
         <v>20</v>
@@ -4232,11 +4263,11 @@
       <c r="E28" s="26" t="s">
         <v>18</v>
       </c>
-      <c r="F28" s="26" t="s">
-        <v>337</v>
+      <c r="F28" s="46" t="s">
+        <v>336</v>
       </c>
       <c r="G28" s="26" t="s">
-        <v>338</v>
+        <v>339</v>
       </c>
       <c r="H28" s="26" t="s">
         <v>38</v>
@@ -4251,66 +4282,66 @@
         <v>43</v>
       </c>
       <c r="L28" s="26" t="s">
-        <v>335</v>
+        <v>49</v>
       </c>
       <c r="M28" s="26" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="N28" s="28">
-        <v>4.8899999999999997</v>
+        <v>2.1</v>
       </c>
       <c r="O28" s="29" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="29" spans="1:15" ht="18" hidden="1" x14ac:dyDescent="0.4">
-      <c r="A29" s="5">
-        <v>2024</v>
-      </c>
-      <c r="B29" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="C29" s="7" t="s">
+    <row r="29" spans="1:15" x14ac:dyDescent="0.4">
+      <c r="A29" s="24">
+        <v>2024</v>
+      </c>
+      <c r="B29" s="25" t="s">
+        <v>138</v>
+      </c>
+      <c r="C29" s="26" t="s">
         <v>20</v>
       </c>
-      <c r="D29" s="7">
-        <v>8</v>
-      </c>
-      <c r="E29" s="7" t="s">
-        <v>26</v>
-      </c>
-      <c r="F29" s="7" t="s">
-        <v>260</v>
-      </c>
-      <c r="G29" s="7" t="s">
-        <v>261</v>
-      </c>
-      <c r="H29" s="7" t="s">
-        <v>64</v>
-      </c>
-      <c r="I29" s="7" t="s">
-        <v>231</v>
-      </c>
-      <c r="J29" s="7" t="s">
+      <c r="D29" s="26">
+        <v>7</v>
+      </c>
+      <c r="E29" s="26" t="s">
+        <v>18</v>
+      </c>
+      <c r="F29" s="26" t="s">
+        <v>337</v>
+      </c>
+      <c r="G29" s="26" t="s">
+        <v>338</v>
+      </c>
+      <c r="H29" s="26" t="s">
+        <v>38</v>
+      </c>
+      <c r="I29" s="26" t="s">
+        <v>40</v>
+      </c>
+      <c r="J29" s="26" t="s">
         <v>11</v>
       </c>
-      <c r="K29" s="10" t="s">
-        <v>262</v>
-      </c>
-      <c r="L29" s="7" t="s">
-        <v>263</v>
-      </c>
-      <c r="M29" s="7" t="s">
-        <v>264</v>
-      </c>
-      <c r="N29" s="9" t="s">
-        <v>123</v>
-      </c>
-      <c r="O29" s="8" t="s">
-        <v>123</v>
-      </c>
-    </row>
-    <row r="30" spans="1:15" hidden="1" x14ac:dyDescent="0.4">
+      <c r="K29" s="27" t="s">
+        <v>43</v>
+      </c>
+      <c r="L29" s="26" t="s">
+        <v>335</v>
+      </c>
+      <c r="M29" s="26" t="s">
+        <v>51</v>
+      </c>
+      <c r="N29" s="28">
+        <v>4.8899999999999997</v>
+      </c>
+      <c r="O29" s="29" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="30" spans="1:15" ht="18" x14ac:dyDescent="0.4">
       <c r="A30" s="5">
         <v>2024</v>
       </c>
@@ -4327,7 +4358,7 @@
         <v>26</v>
       </c>
       <c r="F30" s="7" t="s">
-        <v>265</v>
+        <v>260</v>
       </c>
       <c r="G30" s="7" t="s">
         <v>261</v>
@@ -4342,22 +4373,22 @@
         <v>11</v>
       </c>
       <c r="K30" s="10" t="s">
-        <v>17</v>
+        <v>262</v>
       </c>
       <c r="L30" s="7" t="s">
-        <v>283</v>
+        <v>263</v>
       </c>
       <c r="M30" s="7" t="s">
-        <v>266</v>
+        <v>264</v>
       </c>
       <c r="N30" s="9" t="s">
         <v>123</v>
       </c>
-      <c r="O30" s="6" t="s">
+      <c r="O30" s="8" t="s">
         <v>123</v>
       </c>
     </row>
-    <row r="31" spans="1:15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="31" spans="1:15" x14ac:dyDescent="0.4">
       <c r="A31" s="5">
         <v>2024</v>
       </c>
@@ -4374,7 +4405,7 @@
         <v>26</v>
       </c>
       <c r="F31" s="7" t="s">
-        <v>270</v>
+        <v>265</v>
       </c>
       <c r="G31" s="7" t="s">
         <v>261</v>
@@ -4383,28 +4414,28 @@
         <v>64</v>
       </c>
       <c r="I31" s="7" t="s">
-        <v>271</v>
+        <v>231</v>
       </c>
       <c r="J31" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="K31" s="8" t="s">
-        <v>272</v>
+      <c r="K31" s="10" t="s">
+        <v>17</v>
       </c>
       <c r="L31" s="7" t="s">
-        <v>273</v>
+        <v>283</v>
       </c>
       <c r="M31" s="7" t="s">
-        <v>274</v>
+        <v>266</v>
       </c>
       <c r="N31" s="9" t="s">
         <v>123</v>
       </c>
       <c r="O31" s="6" t="s">
-        <v>275</v>
-      </c>
-    </row>
-    <row r="32" spans="1:15" hidden="1" x14ac:dyDescent="0.4">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="32" spans="1:15" x14ac:dyDescent="0.4">
       <c r="A32" s="5">
         <v>2024</v>
       </c>
@@ -4421,7 +4452,7 @@
         <v>26</v>
       </c>
       <c r="F32" s="7" t="s">
-        <v>276</v>
+        <v>270</v>
       </c>
       <c r="G32" s="7" t="s">
         <v>261</v>
@@ -4430,101 +4461,101 @@
         <v>64</v>
       </c>
       <c r="I32" s="7" t="s">
-        <v>231</v>
+        <v>271</v>
       </c>
       <c r="J32" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="K32" s="10" t="s">
-        <v>123</v>
+      <c r="K32" s="8" t="s">
+        <v>272</v>
       </c>
       <c r="L32" s="7" t="s">
-        <v>278</v>
+        <v>273</v>
       </c>
       <c r="M32" s="7" t="s">
-        <v>277</v>
+        <v>274</v>
       </c>
       <c r="N32" s="9" t="s">
         <v>123</v>
       </c>
       <c r="O32" s="6" t="s">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="33" spans="1:15" x14ac:dyDescent="0.4">
+      <c r="A33" s="5">
+        <v>2024</v>
+      </c>
+      <c r="B33" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="C33" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="D33" s="7">
+        <v>8</v>
+      </c>
+      <c r="E33" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="F33" s="7" t="s">
+        <v>276</v>
+      </c>
+      <c r="G33" s="7" t="s">
+        <v>261</v>
+      </c>
+      <c r="H33" s="7" t="s">
+        <v>64</v>
+      </c>
+      <c r="I33" s="7" t="s">
+        <v>231</v>
+      </c>
+      <c r="J33" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="K33" s="10" t="s">
+        <v>123</v>
+      </c>
+      <c r="L33" s="7" t="s">
+        <v>278</v>
+      </c>
+      <c r="M33" s="7" t="s">
+        <v>277</v>
+      </c>
+      <c r="N33" s="9" t="s">
+        <v>123</v>
+      </c>
+      <c r="O33" s="6" t="s">
         <v>279</v>
       </c>
     </row>
-    <row r="33" spans="1:15" hidden="1" x14ac:dyDescent="0.4">
-      <c r="A33" s="24">
-        <v>2024</v>
-      </c>
-      <c r="B33" s="25" t="s">
+    <row r="34" spans="1:15" x14ac:dyDescent="0.4">
+      <c r="A34" s="24">
+        <v>2024</v>
+      </c>
+      <c r="B34" s="25" t="s">
         <v>123</v>
       </c>
-      <c r="C33" s="26" t="s">
+      <c r="C34" s="26" t="s">
         <v>20</v>
       </c>
-      <c r="D33" s="26">
+      <c r="D34" s="26">
         <v>9</v>
       </c>
-      <c r="E33" s="26" t="s">
+      <c r="E34" s="26" t="s">
         <v>27</v>
       </c>
-      <c r="F33" s="26" t="s">
+      <c r="F34" s="26" t="s">
         <v>250</v>
       </c>
-      <c r="G33" s="26" t="s">
+      <c r="G34" s="26" t="s">
         <v>251</v>
       </c>
-      <c r="H33" s="26" t="s">
+      <c r="H34" s="26" t="s">
         <v>252</v>
       </c>
-      <c r="I33" s="26" t="s">
+      <c r="I34" s="26" t="s">
         <v>182</v>
-      </c>
-      <c r="J33" s="26" t="s">
-        <v>11</v>
-      </c>
-      <c r="K33" s="27" t="s">
-        <v>12</v>
-      </c>
-      <c r="L33" s="26" t="s">
-        <v>253</v>
-      </c>
-      <c r="M33" s="26" t="s">
-        <v>254</v>
-      </c>
-      <c r="N33" s="30">
-        <v>45</v>
-      </c>
-      <c r="O33" s="29" t="s">
-        <v>255</v>
-      </c>
-    </row>
-    <row r="34" spans="1:15" hidden="1" x14ac:dyDescent="0.4">
-      <c r="A34" s="24">
-        <v>2024</v>
-      </c>
-      <c r="B34" s="25" t="s">
-        <v>333</v>
-      </c>
-      <c r="C34" s="26" t="s">
-        <v>28</v>
-      </c>
-      <c r="D34" s="26">
-        <v>10</v>
-      </c>
-      <c r="E34" s="26" t="s">
-        <v>29</v>
-      </c>
-      <c r="F34" s="26" t="s">
-        <v>164</v>
-      </c>
-      <c r="G34" s="26" t="s">
-        <v>198</v>
-      </c>
-      <c r="H34" s="26" t="s">
-        <v>64</v>
-      </c>
-      <c r="I34" s="26" t="s">
-        <v>166</v>
       </c>
       <c r="J34" s="26" t="s">
         <v>11</v>
@@ -4533,24 +4564,24 @@
         <v>12</v>
       </c>
       <c r="L34" s="26" t="s">
-        <v>167</v>
+        <v>253</v>
       </c>
       <c r="M34" s="26" t="s">
-        <v>169</v>
-      </c>
-      <c r="N34" s="28">
-        <v>82.11</v>
+        <v>254</v>
+      </c>
+      <c r="N34" s="30">
+        <v>45</v>
       </c>
       <c r="O34" s="29" t="s">
-        <v>171</v>
-      </c>
-    </row>
-    <row r="35" spans="1:15" hidden="1" x14ac:dyDescent="0.4">
+        <v>255</v>
+      </c>
+    </row>
+    <row r="35" spans="1:15" x14ac:dyDescent="0.4">
       <c r="A35" s="24">
         <v>2024</v>
       </c>
       <c r="B35" s="25" t="s">
-        <v>334</v>
+        <v>333</v>
       </c>
       <c r="C35" s="26" t="s">
         <v>28</v>
@@ -4562,7 +4593,7 @@
         <v>29</v>
       </c>
       <c r="F35" s="26" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="G35" s="26" t="s">
         <v>198</v>
@@ -4580,66 +4611,66 @@
         <v>12</v>
       </c>
       <c r="L35" s="26" t="s">
+        <v>167</v>
+      </c>
+      <c r="M35" s="26" t="s">
+        <v>169</v>
+      </c>
+      <c r="N35" s="28">
+        <v>82.11</v>
+      </c>
+      <c r="O35" s="29" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="36" spans="1:15" x14ac:dyDescent="0.4">
+      <c r="A36" s="24">
+        <v>2024</v>
+      </c>
+      <c r="B36" s="25" t="s">
+        <v>334</v>
+      </c>
+      <c r="C36" s="26" t="s">
+        <v>28</v>
+      </c>
+      <c r="D36" s="26">
+        <v>10</v>
+      </c>
+      <c r="E36" s="26" t="s">
+        <v>29</v>
+      </c>
+      <c r="F36" s="26" t="s">
+        <v>165</v>
+      </c>
+      <c r="G36" s="26" t="s">
+        <v>198</v>
+      </c>
+      <c r="H36" s="26" t="s">
+        <v>64</v>
+      </c>
+      <c r="I36" s="26" t="s">
+        <v>166</v>
+      </c>
+      <c r="J36" s="26" t="s">
+        <v>11</v>
+      </c>
+      <c r="K36" s="27" t="s">
+        <v>12</v>
+      </c>
+      <c r="L36" s="26" t="s">
         <v>168</v>
       </c>
-      <c r="M35" s="26" t="s">
+      <c r="M36" s="26" t="s">
         <v>170</v>
       </c>
-      <c r="N35" s="28">
+      <c r="N36" s="28">
         <v>17.89</v>
       </c>
-      <c r="O35" s="29" t="s">
+      <c r="O36" s="29" t="s">
         <v>172</v>
       </c>
     </row>
-    <row r="36" spans="1:15" hidden="1" x14ac:dyDescent="0.4">
-      <c r="A36" s="18">
-        <v>2024</v>
-      </c>
-      <c r="B36" s="19" t="s">
-        <v>123</v>
-      </c>
-      <c r="C36" s="20" t="s">
-        <v>28</v>
-      </c>
-      <c r="D36" s="20">
-        <v>11</v>
-      </c>
-      <c r="E36" s="20" t="s">
-        <v>215</v>
-      </c>
-      <c r="F36" s="20" t="s">
-        <v>123</v>
-      </c>
-      <c r="G36" s="20" t="s">
-        <v>123</v>
-      </c>
-      <c r="H36" s="20" t="s">
-        <v>123</v>
-      </c>
-      <c r="I36" s="20" t="s">
-        <v>123</v>
-      </c>
-      <c r="J36" s="20" t="s">
-        <v>123</v>
-      </c>
-      <c r="K36" s="21" t="s">
-        <v>123</v>
-      </c>
-      <c r="L36" s="20" t="s">
-        <v>123</v>
-      </c>
-      <c r="M36" s="20" t="s">
-        <v>123</v>
-      </c>
-      <c r="N36" s="22" t="s">
-        <v>123</v>
-      </c>
-      <c r="O36" s="23" t="s">
-        <v>123</v>
-      </c>
-    </row>
-    <row r="37" spans="1:15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="37" spans="1:15" x14ac:dyDescent="0.4">
       <c r="A37" s="18">
         <v>2024</v>
       </c>
@@ -4650,10 +4681,10 @@
         <v>28</v>
       </c>
       <c r="D37" s="20">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="E37" s="20" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="F37" s="20" t="s">
         <v>123</v>
@@ -4686,59 +4717,59 @@
         <v>123</v>
       </c>
     </row>
-    <row r="38" spans="1:15" hidden="1" x14ac:dyDescent="0.4">
-      <c r="A38" s="24">
-        <v>2024</v>
-      </c>
-      <c r="B38" s="25" t="s">
+    <row r="38" spans="1:15" x14ac:dyDescent="0.4">
+      <c r="A38" s="18">
+        <v>2024</v>
+      </c>
+      <c r="B38" s="19" t="s">
+        <v>123</v>
+      </c>
+      <c r="C38" s="20" t="s">
+        <v>28</v>
+      </c>
+      <c r="D38" s="20">
+        <v>12</v>
+      </c>
+      <c r="E38" s="20" t="s">
+        <v>216</v>
+      </c>
+      <c r="F38" s="20" t="s">
+        <v>123</v>
+      </c>
+      <c r="G38" s="20" t="s">
+        <v>123</v>
+      </c>
+      <c r="H38" s="20" t="s">
+        <v>123</v>
+      </c>
+      <c r="I38" s="20" t="s">
+        <v>123</v>
+      </c>
+      <c r="J38" s="20" t="s">
+        <v>123</v>
+      </c>
+      <c r="K38" s="21" t="s">
+        <v>123</v>
+      </c>
+      <c r="L38" s="20" t="s">
+        <v>123</v>
+      </c>
+      <c r="M38" s="20" t="s">
+        <v>123</v>
+      </c>
+      <c r="N38" s="22" t="s">
+        <v>123</v>
+      </c>
+      <c r="O38" s="23" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="39" spans="1:15" x14ac:dyDescent="0.4">
+      <c r="A39" s="24">
+        <v>2024</v>
+      </c>
+      <c r="B39" s="25" t="s">
         <v>86</v>
-      </c>
-      <c r="C38" s="26" t="s">
-        <v>28</v>
-      </c>
-      <c r="D38" s="26">
-        <v>13</v>
-      </c>
-      <c r="E38" s="26" t="s">
-        <v>30</v>
-      </c>
-      <c r="F38" s="26" t="s">
-        <v>87</v>
-      </c>
-      <c r="G38" s="26" t="s">
-        <v>217</v>
-      </c>
-      <c r="H38" s="26" t="s">
-        <v>82</v>
-      </c>
-      <c r="I38" s="26" t="s">
-        <v>90</v>
-      </c>
-      <c r="J38" s="26" t="s">
-        <v>11</v>
-      </c>
-      <c r="K38" s="27" t="s">
-        <v>88</v>
-      </c>
-      <c r="L38" s="26" t="s">
-        <v>89</v>
-      </c>
-      <c r="M38" s="26" t="s">
-        <v>111</v>
-      </c>
-      <c r="N38" s="28">
-        <v>49.16</v>
-      </c>
-      <c r="O38" s="29" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="39" spans="1:15" hidden="1" x14ac:dyDescent="0.4">
-      <c r="A39" s="24">
-        <v>2024</v>
-      </c>
-      <c r="B39" s="25" t="s">
-        <v>100</v>
       </c>
       <c r="C39" s="26" t="s">
         <v>28</v>
@@ -4750,42 +4781,42 @@
         <v>30</v>
       </c>
       <c r="F39" s="26" t="s">
-        <v>95</v>
+        <v>87</v>
       </c>
       <c r="G39" s="26" t="s">
-        <v>197</v>
+        <v>217</v>
       </c>
       <c r="H39" s="26" t="s">
-        <v>92</v>
+        <v>82</v>
       </c>
       <c r="I39" s="26" t="s">
-        <v>106</v>
+        <v>90</v>
       </c>
       <c r="J39" s="26" t="s">
         <v>11</v>
       </c>
       <c r="K39" s="27" t="s">
-        <v>12</v>
+        <v>88</v>
       </c>
       <c r="L39" s="26" t="s">
-        <v>94</v>
+        <v>89</v>
       </c>
       <c r="M39" s="26" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="N39" s="28">
-        <v>37.65</v>
-      </c>
-      <c r="O39" s="43" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="40" spans="1:15" hidden="1" x14ac:dyDescent="0.4">
+        <v>49.16</v>
+      </c>
+      <c r="O39" s="29" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="40" spans="1:15" x14ac:dyDescent="0.4">
       <c r="A40" s="24">
         <v>2024</v>
       </c>
       <c r="B40" s="25" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="C40" s="26" t="s">
         <v>28</v>
@@ -4797,7 +4828,7 @@
         <v>30</v>
       </c>
       <c r="F40" s="26" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="G40" s="26" t="s">
         <v>197</v>
@@ -4815,24 +4846,24 @@
         <v>12</v>
       </c>
       <c r="L40" s="26" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="M40" s="26" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="N40" s="28">
-        <v>32.590000000000003</v>
+        <v>37.65</v>
       </c>
       <c r="O40" s="43" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="41" spans="1:15" hidden="1" x14ac:dyDescent="0.4">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="41" spans="1:15" x14ac:dyDescent="0.4">
       <c r="A41" s="24">
         <v>2024</v>
       </c>
       <c r="B41" s="25" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="C41" s="26" t="s">
         <v>28</v>
@@ -4844,16 +4875,16 @@
         <v>30</v>
       </c>
       <c r="F41" s="26" t="s">
-        <v>103</v>
+        <v>96</v>
       </c>
       <c r="G41" s="26" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="H41" s="26" t="s">
-        <v>104</v>
+        <v>92</v>
       </c>
       <c r="I41" s="26" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="J41" s="26" t="s">
         <v>11</v>
@@ -4862,45 +4893,45 @@
         <v>12</v>
       </c>
       <c r="L41" s="26" t="s">
-        <v>107</v>
+        <v>97</v>
       </c>
       <c r="M41" s="26" t="s">
-        <v>108</v>
-      </c>
-      <c r="N41" s="30">
-        <v>70</v>
-      </c>
-      <c r="O41" s="31" t="s">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="42" spans="1:15" hidden="1" x14ac:dyDescent="0.4">
+        <v>109</v>
+      </c>
+      <c r="N41" s="28">
+        <v>32.590000000000003</v>
+      </c>
+      <c r="O41" s="43" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="42" spans="1:15" x14ac:dyDescent="0.4">
       <c r="A42" s="24">
         <v>2024</v>
       </c>
       <c r="B42" s="25" t="s">
-        <v>225</v>
+        <v>102</v>
       </c>
       <c r="C42" s="26" t="s">
         <v>28</v>
       </c>
       <c r="D42" s="26">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E42" s="26" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="F42" s="26" t="s">
-        <v>193</v>
+        <v>103</v>
       </c>
       <c r="G42" s="26" t="s">
-        <v>227</v>
+        <v>196</v>
       </c>
       <c r="H42" s="26" t="s">
-        <v>181</v>
+        <v>104</v>
       </c>
       <c r="I42" s="26" t="s">
-        <v>182</v>
+        <v>105</v>
       </c>
       <c r="J42" s="26" t="s">
         <v>11</v>
@@ -4909,45 +4940,45 @@
         <v>12</v>
       </c>
       <c r="L42" s="26" t="s">
-        <v>192</v>
+        <v>107</v>
       </c>
       <c r="M42" s="26" t="s">
-        <v>229</v>
+        <v>108</v>
       </c>
       <c r="N42" s="30">
-        <v>18</v>
-      </c>
-      <c r="O42" s="29" t="s">
-        <v>230</v>
-      </c>
-    </row>
-    <row r="43" spans="1:15" hidden="1" x14ac:dyDescent="0.4">
+        <v>70</v>
+      </c>
+      <c r="O42" s="31" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="43" spans="1:15" x14ac:dyDescent="0.4">
       <c r="A43" s="24">
         <v>2024</v>
       </c>
       <c r="B43" s="25" t="s">
-        <v>218</v>
+        <v>225</v>
       </c>
       <c r="C43" s="26" t="s">
         <v>28</v>
       </c>
       <c r="D43" s="26">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="E43" s="26" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="F43" s="26" t="s">
-        <v>223</v>
+        <v>193</v>
       </c>
       <c r="G43" s="26" t="s">
-        <v>195</v>
+        <v>227</v>
       </c>
       <c r="H43" s="26" t="s">
-        <v>64</v>
+        <v>181</v>
       </c>
       <c r="I43" s="26" t="s">
-        <v>120</v>
+        <v>182</v>
       </c>
       <c r="J43" s="26" t="s">
         <v>11</v>
@@ -4956,24 +4987,24 @@
         <v>12</v>
       </c>
       <c r="L43" s="26" t="s">
-        <v>121</v>
+        <v>192</v>
       </c>
       <c r="M43" s="26" t="s">
-        <v>220</v>
+        <v>229</v>
       </c>
       <c r="N43" s="30">
-        <v>94</v>
+        <v>18</v>
       </c>
       <c r="O43" s="29" t="s">
-        <v>224</v>
-      </c>
-    </row>
-    <row r="44" spans="1:15" hidden="1" x14ac:dyDescent="0.4">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="44" spans="1:15" x14ac:dyDescent="0.4">
       <c r="A44" s="24">
         <v>2024</v>
       </c>
       <c r="B44" s="25" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="C44" s="26" t="s">
         <v>28</v>
@@ -4985,7 +5016,7 @@
         <v>32</v>
       </c>
       <c r="F44" s="26" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="G44" s="26" t="s">
         <v>195</v>
@@ -5006,21 +5037,21 @@
         <v>121</v>
       </c>
       <c r="M44" s="26" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="N44" s="30">
-        <v>6</v>
+        <v>94</v>
       </c>
       <c r="O44" s="29" t="s">
         <v>224</v>
       </c>
     </row>
-    <row r="45" spans="1:15" hidden="1" x14ac:dyDescent="0.4">
+    <row r="45" spans="1:15" x14ac:dyDescent="0.4">
       <c r="A45" s="24">
         <v>2024</v>
       </c>
       <c r="B45" s="25" t="s">
-        <v>119</v>
+        <v>219</v>
       </c>
       <c r="C45" s="26" t="s">
         <v>28</v>
@@ -5032,7 +5063,7 @@
         <v>32</v>
       </c>
       <c r="F45" s="26" t="s">
-        <v>132</v>
+        <v>222</v>
       </c>
       <c r="G45" s="26" t="s">
         <v>195</v>
@@ -5047,25 +5078,27 @@
         <v>11</v>
       </c>
       <c r="K45" s="27" t="s">
-        <v>122</v>
+        <v>12</v>
       </c>
       <c r="L45" s="26" t="s">
-        <v>133</v>
-      </c>
-      <c r="M45" s="26"/>
-      <c r="N45" s="32">
-        <v>737000000</v>
+        <v>121</v>
+      </c>
+      <c r="M45" s="26" t="s">
+        <v>221</v>
+      </c>
+      <c r="N45" s="30">
+        <v>6</v>
       </c>
       <c r="O45" s="29" t="s">
-        <v>134</v>
-      </c>
-    </row>
-    <row r="46" spans="1:15" hidden="1" x14ac:dyDescent="0.4">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="46" spans="1:15" x14ac:dyDescent="0.4">
       <c r="A46" s="24">
         <v>2024</v>
       </c>
       <c r="B46" s="25" t="s">
-        <v>125</v>
+        <v>119</v>
       </c>
       <c r="C46" s="26" t="s">
         <v>28</v>
@@ -5077,7 +5110,7 @@
         <v>32</v>
       </c>
       <c r="F46" s="26" t="s">
-        <v>126</v>
+        <v>132</v>
       </c>
       <c r="G46" s="26" t="s">
         <v>195</v>
@@ -5095,24 +5128,22 @@
         <v>122</v>
       </c>
       <c r="L46" s="26" t="s">
-        <v>128</v>
-      </c>
-      <c r="M46" s="26" t="s">
-        <v>130</v>
-      </c>
+        <v>133</v>
+      </c>
+      <c r="M46" s="26"/>
       <c r="N46" s="32">
-        <v>575000000</v>
+        <v>737000000</v>
       </c>
       <c r="O46" s="29" t="s">
-        <v>135</v>
-      </c>
-    </row>
-    <row r="47" spans="1:15" hidden="1" x14ac:dyDescent="0.4">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="47" spans="1:15" x14ac:dyDescent="0.4">
       <c r="A47" s="24">
         <v>2024</v>
       </c>
       <c r="B47" s="25" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="C47" s="26" t="s">
         <v>28</v>
@@ -5124,7 +5155,7 @@
         <v>32</v>
       </c>
       <c r="F47" s="26" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="G47" s="26" t="s">
         <v>195</v>
@@ -5142,66 +5173,66 @@
         <v>122</v>
       </c>
       <c r="L47" s="26" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="M47" s="26" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="N47" s="32">
-        <v>162000000</v>
+        <v>575000000</v>
       </c>
       <c r="O47" s="29" t="s">
         <v>135</v>
       </c>
     </row>
-    <row r="48" spans="1:15" ht="16.8" hidden="1" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A48" s="5">
-        <v>2024</v>
-      </c>
-      <c r="B48" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="C48" s="7" t="s">
+    <row r="48" spans="1:15" x14ac:dyDescent="0.4">
+      <c r="A48" s="24">
+        <v>2024</v>
+      </c>
+      <c r="B48" s="25" t="s">
+        <v>124</v>
+      </c>
+      <c r="C48" s="26" t="s">
         <v>28</v>
       </c>
-      <c r="D48" s="7">
-        <v>16</v>
-      </c>
-      <c r="E48" s="7" t="s">
-        <v>33</v>
-      </c>
-      <c r="F48" s="7" t="s">
-        <v>244</v>
-      </c>
-      <c r="G48" s="7" t="s">
-        <v>241</v>
-      </c>
-      <c r="H48" s="7" t="s">
-        <v>242</v>
-      </c>
-      <c r="I48" s="7" t="s">
-        <v>246</v>
-      </c>
-      <c r="J48" s="7" t="s">
+      <c r="D48" s="26">
+        <v>15</v>
+      </c>
+      <c r="E48" s="26" t="s">
+        <v>32</v>
+      </c>
+      <c r="F48" s="26" t="s">
+        <v>127</v>
+      </c>
+      <c r="G48" s="26" t="s">
+        <v>195</v>
+      </c>
+      <c r="H48" s="26" t="s">
+        <v>64</v>
+      </c>
+      <c r="I48" s="26" t="s">
+        <v>120</v>
+      </c>
+      <c r="J48" s="26" t="s">
         <v>11</v>
       </c>
-      <c r="K48" s="10" t="s">
-        <v>123</v>
-      </c>
-      <c r="L48" s="12" t="s">
-        <v>247</v>
-      </c>
-      <c r="M48" s="7" t="s">
-        <v>243</v>
-      </c>
-      <c r="N48" s="9" t="s">
-        <v>123</v>
-      </c>
-      <c r="O48" s="8" t="s">
-        <v>249</v>
-      </c>
-    </row>
-    <row r="49" spans="1:15" ht="16.8" hidden="1" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="K48" s="27" t="s">
+        <v>122</v>
+      </c>
+      <c r="L48" s="26" t="s">
+        <v>129</v>
+      </c>
+      <c r="M48" s="26" t="s">
+        <v>131</v>
+      </c>
+      <c r="N48" s="32">
+        <v>162000000</v>
+      </c>
+      <c r="O48" s="29" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="49" spans="1:15" ht="16.8" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A49" s="5">
         <v>2024</v>
       </c>
@@ -5218,7 +5249,7 @@
         <v>33</v>
       </c>
       <c r="F49" s="7" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="G49" s="7" t="s">
         <v>241</v>
@@ -5233,118 +5264,118 @@
         <v>11</v>
       </c>
       <c r="K49" s="10" t="s">
-        <v>17</v>
+        <v>123</v>
       </c>
       <c r="L49" s="12" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="M49" s="7" t="s">
         <v>243</v>
       </c>
-      <c r="N49" s="9"/>
+      <c r="N49" s="9" t="s">
+        <v>123</v>
+      </c>
       <c r="O49" s="8" t="s">
         <v>249</v>
       </c>
     </row>
-    <row r="50" spans="1:15" hidden="1" x14ac:dyDescent="0.4">
-      <c r="A50" s="24">
-        <v>2024</v>
-      </c>
-      <c r="B50" s="25" t="s">
+    <row r="50" spans="1:15" ht="16.8" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A50" s="5">
+        <v>2024</v>
+      </c>
+      <c r="B50" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="C50" s="7" t="s">
+        <v>28</v>
+      </c>
+      <c r="D50" s="7">
+        <v>16</v>
+      </c>
+      <c r="E50" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="F50" s="7" t="s">
+        <v>245</v>
+      </c>
+      <c r="G50" s="7" t="s">
+        <v>241</v>
+      </c>
+      <c r="H50" s="7" t="s">
+        <v>242</v>
+      </c>
+      <c r="I50" s="7" t="s">
+        <v>246</v>
+      </c>
+      <c r="J50" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="K50" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="L50" s="12" t="s">
+        <v>248</v>
+      </c>
+      <c r="M50" s="7" t="s">
+        <v>243</v>
+      </c>
+      <c r="N50" s="9"/>
+      <c r="O50" s="8" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="51" spans="1:15" x14ac:dyDescent="0.4">
+      <c r="A51" s="24">
+        <v>2024</v>
+      </c>
+      <c r="B51" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="C50" s="26" t="s">
+      <c r="C51" s="26" t="s">
         <v>28</v>
       </c>
-      <c r="D50" s="26">
+      <c r="D51" s="26">
         <v>17</v>
       </c>
-      <c r="E50" s="26" t="s">
+      <c r="E51" s="26" t="s">
         <v>34</v>
       </c>
-      <c r="F50" s="26" t="s">
+      <c r="F51" s="26" t="s">
         <v>226</v>
       </c>
-      <c r="G50" s="26" t="s">
+      <c r="G51" s="26" t="s">
         <v>194</v>
       </c>
-      <c r="H50" s="26" t="s">
+      <c r="H51" s="26" t="s">
         <v>181</v>
       </c>
-      <c r="I50" s="26" t="s">
+      <c r="I51" s="26" t="s">
         <v>182</v>
       </c>
-      <c r="J50" s="26" t="s">
+      <c r="J51" s="26" t="s">
         <v>11</v>
       </c>
-      <c r="K50" s="27" t="s">
+      <c r="K51" s="27" t="s">
         <v>12</v>
       </c>
-      <c r="L50" s="26" t="s">
+      <c r="L51" s="26" t="s">
         <v>228</v>
       </c>
-      <c r="M50" s="26" t="s">
+      <c r="M51" s="26" t="s">
         <v>210</v>
       </c>
-      <c r="N50" s="30">
+      <c r="N51" s="30">
         <v>9</v>
       </c>
-      <c r="O50" s="29" t="s">
+      <c r="O51" s="29" t="s">
         <v>230</v>
       </c>
     </row>
-    <row r="51" spans="1:15" hidden="1" x14ac:dyDescent="0.4">
-      <c r="A51" s="5">
-        <v>2024</v>
-      </c>
-      <c r="B51" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="C51" s="7" t="s">
-        <v>28</v>
-      </c>
-      <c r="D51" s="7">
-        <v>18</v>
-      </c>
-      <c r="E51" s="7" t="s">
-        <v>35</v>
-      </c>
-      <c r="F51" s="7" t="s">
-        <v>256</v>
-      </c>
-      <c r="G51" s="7" t="s">
-        <v>241</v>
-      </c>
-      <c r="H51" s="7" t="s">
-        <v>64</v>
-      </c>
-      <c r="I51" s="7" t="s">
-        <v>166</v>
-      </c>
-      <c r="J51" s="7" t="s">
-        <v>11</v>
-      </c>
-      <c r="K51" s="10" t="s">
-        <v>12</v>
-      </c>
-      <c r="L51" s="7" t="s">
-        <v>257</v>
-      </c>
-      <c r="M51" s="7" t="s">
-        <v>258</v>
-      </c>
-      <c r="N51" s="9" t="s">
-        <v>123</v>
-      </c>
-      <c r="O51" s="8" t="s">
-        <v>259</v>
-      </c>
-    </row>
-    <row r="52" spans="1:15" hidden="1" x14ac:dyDescent="0.4">
-      <c r="A52" s="13">
-        <v>2024</v>
-      </c>
-      <c r="B52" s="14" t="s">
+    <row r="52" spans="1:15" x14ac:dyDescent="0.4">
+      <c r="A52" s="5">
+        <v>2024</v>
+      </c>
+      <c r="B52" s="6" t="s">
         <v>123</v>
       </c>
       <c r="C52" s="7" t="s">
@@ -5356,8 +5387,8 @@
       <c r="E52" s="7" t="s">
         <v>35</v>
       </c>
-      <c r="F52" s="15" t="s">
-        <v>267</v>
+      <c r="F52" s="7" t="s">
+        <v>256</v>
       </c>
       <c r="G52" s="7" t="s">
         <v>241</v>
@@ -5374,16 +5405,63 @@
       <c r="K52" s="10" t="s">
         <v>12</v>
       </c>
-      <c r="L52" s="15" t="s">
+      <c r="L52" s="7" t="s">
+        <v>257</v>
+      </c>
+      <c r="M52" s="7" t="s">
+        <v>258</v>
+      </c>
+      <c r="N52" s="9" t="s">
+        <v>123</v>
+      </c>
+      <c r="O52" s="8" t="s">
+        <v>259</v>
+      </c>
+    </row>
+    <row r="53" spans="1:15" x14ac:dyDescent="0.4">
+      <c r="A53" s="13">
+        <v>2024</v>
+      </c>
+      <c r="B53" s="14" t="s">
+        <v>123</v>
+      </c>
+      <c r="C53" s="7" t="s">
+        <v>28</v>
+      </c>
+      <c r="D53" s="7">
+        <v>18</v>
+      </c>
+      <c r="E53" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="F53" s="15" t="s">
+        <v>267</v>
+      </c>
+      <c r="G53" s="7" t="s">
+        <v>241</v>
+      </c>
+      <c r="H53" s="7" t="s">
+        <v>64</v>
+      </c>
+      <c r="I53" s="7" t="s">
+        <v>166</v>
+      </c>
+      <c r="J53" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="K53" s="10" t="s">
+        <v>12</v>
+      </c>
+      <c r="L53" s="15" t="s">
         <v>268</v>
       </c>
-      <c r="M52" s="15" t="s">
+      <c r="M53" s="15" t="s">
         <v>269</v>
       </c>
-      <c r="N52" s="16" t="s">
+      <c r="N53" s="16" t="s">
         <v>123</v>
       </c>
-      <c r="O52" s="8" t="s">
+      <c r="O53" s="8" t="s">
         <v>259</v>
       </c>
     </row>
@@ -5391,7 +5469,7 @@
   <phoneticPr fontId="5" type="noConversion"/>
   <hyperlinks>
     <hyperlink ref="O13" r:id="rId1" display="https://www.seg-social.es/wps/portal/wss/internet/EstadisticasPresupuestosEstudios/Estadisticas/EST8/EST10/EST305/c43ad8ea-fe79-4329-ac8e-e5758f3c4d7a/f83fe4aa-2dee-49c5-8317-98d105813796" xr:uid="{61128FB4-53B2-4EAF-8DD6-669E31DEF896}"/>
-    <hyperlink ref="O40" r:id="rId2" display="https://www.seg-social.es/wps/portal/wss/internet/EstadisticasPresupuestosEstudios/Estadisticas/EST8/EST10/EST305/c43ad8ea-fe79-4329-ac8e-e5758f3c4d7a/f83fe4aa-2dee-49c5-8317-98d105813796" xr:uid="{AAB67715-CF03-4157-B01F-134351755964}"/>
+    <hyperlink ref="O41" r:id="rId2" display="https://www.seg-social.es/wps/portal/wss/internet/EstadisticasPresupuestosEstudios/Estadisticas/EST8/EST10/EST305/c43ad8ea-fe79-4329-ac8e-e5758f3c4d7a/f83fe4aa-2dee-49c5-8317-98d105813796" xr:uid="{AAB67715-CF03-4157-B01F-134351755964}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <legacyDrawing r:id="rId3"/>
@@ -5460,10 +5538,12 @@
         <v>26001</v>
       </c>
       <c r="G2" s="36">
-        <v>5.4483715378038751</v>
+        <f>Turistas[[#This Row],[1. Turistas extranjeros que visitaron Calp]]/Turistas[[#This Row],[1. Total turistas]]</f>
+        <v>0.5195954001769163</v>
       </c>
       <c r="H2" s="36">
-        <v>4.0201603429575581</v>
+        <f>Turistas[[#This Row],[1. Turistas nacionales que visitaron Calp]]/Turistas[[#This Row],[1. Total turistas]]</f>
+        <v>0.4804045998230837</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -5486,10 +5566,12 @@
         <v>23273</v>
       </c>
       <c r="G3" s="36">
-        <v>5.1955122517784842</v>
+        <f>Turistas[[#This Row],[1. Turistas extranjeros que visitaron Calp]]/Turistas[[#This Row],[1. Total turistas]]</f>
+        <v>0.55355991921969661</v>
       </c>
       <c r="H3" s="36">
-        <v>3.3439649318172311</v>
+        <f>Turistas[[#This Row],[1. Turistas nacionales que visitaron Calp]]/Turistas[[#This Row],[1. Total turistas]]</f>
+        <v>0.44644008078030334</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.3">
@@ -5512,10 +5594,12 @@
         <v>33487</v>
       </c>
       <c r="G4" s="36">
-        <v>6.4831991740736559</v>
+        <f>Turistas[[#This Row],[1. Turistas extranjeros que visitaron Calp]]/Turistas[[#This Row],[1. Total turistas]]</f>
+        <v>0.4800668916295876</v>
       </c>
       <c r="H4" s="36">
-        <v>5.6036355560991149</v>
+        <f>Turistas[[#This Row],[1. Turistas nacionales que visitaron Calp]]/Turistas[[#This Row],[1. Total turistas]]</f>
+        <v>0.5199331083704124</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.3">
@@ -5538,10 +5622,12 @@
         <v>38995</v>
       </c>
       <c r="G5" s="36">
-        <v>7.8200867867916308</v>
+        <f>Turistas[[#This Row],[1. Turistas extranjeros que visitaron Calp]]/Turistas[[#This Row],[1. Total turistas]]</f>
+        <v>0.49726888062572122</v>
       </c>
       <c r="H5" s="36">
-        <v>6.3094406663469673</v>
+        <f>Turistas[[#This Row],[1. Turistas nacionales que visitaron Calp]]/Turistas[[#This Row],[1. Total turistas]]</f>
+        <v>0.50273111937427872</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.3">
@@ -5564,10 +5650,12 @@
         <v>44339</v>
       </c>
       <c r="G6" s="36">
-        <v>8.8262812343727308</v>
+        <f>Turistas[[#This Row],[1. Turistas extranjeros que visitaron Calp]]/Turistas[[#This Row],[1. Total turistas]]</f>
+        <v>0.49360608042581022</v>
       </c>
       <c r="H6" s="36">
-        <v>7.2263758050136948</v>
+        <f>Turistas[[#This Row],[1. Turistas nacionales que visitaron Calp]]/Turistas[[#This Row],[1. Total turistas]]</f>
+        <v>0.50639391957418978</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.3">
@@ -5590,10 +5678,12 @@
         <v>54257</v>
       </c>
       <c r="G7" s="36">
-        <v>9.5949412011421007</v>
+        <f>Turistas[[#This Row],[1. Turistas extranjeros que visitaron Calp]]/Turistas[[#This Row],[1. Total turistas]]</f>
+        <v>0.43850563060987524</v>
       </c>
       <c r="H7" s="36">
-        <v>9.804994383812506</v>
+        <f>Turistas[[#This Row],[1. Turistas nacionales que visitaron Calp]]/Turistas[[#This Row],[1. Total turistas]]</f>
+        <v>0.56149436939012476</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.3">
@@ -5616,10 +5706,12 @@
         <v>84458</v>
       </c>
       <c r="G8" s="36">
-        <v>11.344791985933442</v>
+        <f>Turistas[[#This Row],[1. Turistas extranjeros que visitaron Calp]]/Turistas[[#This Row],[1. Total turistas]]</f>
+        <v>0.33307679556702741</v>
       </c>
       <c r="H8" s="36">
-        <v>18.128538278582209</v>
+        <f>Turistas[[#This Row],[1. Turistas nacionales que visitaron Calp]]/Turistas[[#This Row],[1. Total turistas]]</f>
+        <v>0.66692320443297259</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.3">
@@ -5642,10 +5734,12 @@
         <v>102065</v>
       </c>
       <c r="G9" s="36">
-        <v>13.44227387846623</v>
+        <f>Turistas[[#This Row],[1. Turistas extranjeros que visitaron Calp]]/Turistas[[#This Row],[1. Total turistas]]</f>
+        <v>0.32657620144025867</v>
       </c>
       <c r="H9" s="36">
-        <v>22.121341834320859</v>
+        <f>Turistas[[#This Row],[1. Turistas nacionales que visitaron Calp]]/Turistas[[#This Row],[1. Total turistas]]</f>
+        <v>0.67342379855974133</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.3">
@@ -5668,10 +5762,12 @@
         <v>61448</v>
       </c>
       <c r="G10" s="36">
-        <v>10.580568146989078</v>
+        <f>Turistas[[#This Row],[1. Turistas extranjeros que visitaron Calp]]/Turistas[[#This Row],[1. Total turistas]]</f>
+        <v>0.42696263507355814</v>
       </c>
       <c r="H10" s="36">
-        <v>11.332790488849696</v>
+        <f>Turistas[[#This Row],[1. Turistas nacionales que visitaron Calp]]/Turistas[[#This Row],[1. Total turistas]]</f>
+        <v>0.57303736492644186</v>
       </c>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.3">
@@ -5694,10 +5790,12 @@
         <v>40356</v>
       </c>
       <c r="G11" s="36">
-        <v>10.694294333048346</v>
+        <f>Turistas[[#This Row],[1. Turistas extranjeros que visitaron Calp]]/Turistas[[#This Row],[1. Total turistas]]</f>
+        <v>0.65710179403310531</v>
       </c>
       <c r="H11" s="36">
-        <v>4.4536849592383874</v>
+        <f>Turistas[[#This Row],[1. Turistas nacionales que visitaron Calp]]/Turistas[[#This Row],[1. Total turistas]]</f>
+        <v>0.34289820596689463</v>
       </c>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.3">
@@ -5720,10 +5818,12 @@
         <v>23984</v>
       </c>
       <c r="G12" s="36">
-        <v>5.7512380829475243</v>
+        <f>Turistas[[#This Row],[1. Turistas extranjeros que visitaron Calp]]/Turistas[[#This Row],[1. Total turistas]]</f>
+        <v>0.59460473649099399</v>
       </c>
       <c r="H12" s="36">
-        <v>3.1292946132876742</v>
+        <f>Turistas[[#This Row],[1. Turistas nacionales que visitaron Calp]]/Turistas[[#This Row],[1. Total turistas]]</f>
+        <v>0.40539526350900601</v>
       </c>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.3">
@@ -5746,10 +5846,12 @@
         <v>26010</v>
       </c>
       <c r="G13" s="36">
-        <v>4.8184413866529017</v>
+        <f>Turistas[[#This Row],[1. Turistas extranjeros que visitaron Calp]]/Turistas[[#This Row],[1. Total turistas]]</f>
+        <v>0.45936178392925797</v>
       </c>
       <c r="H13" s="36">
-        <v>4.5257781396741006</v>
+        <f>Turistas[[#This Row],[1. Turistas nacionales que visitaron Calp]]/Turistas[[#This Row],[1. Total turistas]]</f>
+        <v>0.54063821607074203</v>
       </c>
     </row>
     <row r="19" spans="9:21" x14ac:dyDescent="0.3">

</xml_diff>